<commit_message>
Fix QA audit issues: Inventory, Sales validation, Taxes, Security roles
</commit_message>
<xml_diff>
--- a/master-assist/server/database.xlsx
+++ b/master-assist/server/database.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
   <si>
     <t>ID</t>
   </si>
@@ -69,6 +69,39 @@
   </si>
   <si>
     <t>TEST1</t>
+  </si>
+  <si>
+    <t>890481650070</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Shoe</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>890685711566</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>Clothing</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>Pcs</t>
+  </si>
+  <si>
+    <t>Inclusive</t>
   </si>
   <si>
     <t>Bill No</t>
@@ -478,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -547,7 +580,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -557,11 +590,97 @@
       <c r="C2" t="s">
         <v>18</v>
       </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
       <c r="E2">
         <v>2</v>
       </c>
       <c r="F2">
         <v>100</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3">
+        <v>499</v>
+      </c>
+      <c r="G3">
+        <v>459</v>
+      </c>
+      <c r="H3">
+        <v>399</v>
+      </c>
+      <c r="I3">
+        <v>50</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" t="s">
+        <v>20</v>
+      </c>
+      <c r="P3" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -587,34 +706,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="H1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="I1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="J1" t="s">
         <v>12</v>
       </c>
       <c r="K1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -622,13 +741,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H2">
         <v>400</v>
       </c>
       <c r="K2" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -636,13 +755,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H3">
         <v>400</v>
       </c>
       <c r="K3" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
QA Automation & Hardware Test Fixes
</commit_message>
<xml_diff>
--- a/master-assist/server/database.xlsx
+++ b/master-assist/server/database.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="60">
   <si>
     <t>ID</t>
   </si>
@@ -104,6 +104,45 @@
     <t>Inclusive</t>
   </si>
   <si>
+    <t>E2E Test Product</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785396388194</t>
+  </si>
+  <si>
+    <t>123456789</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785396438199</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785396461066</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785396486126</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785396570404</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785398604451</t>
+  </si>
+  <si>
+    <t>E2E-SKU-1785398779711</t>
+  </si>
+  <si>
+    <t>Atta 5kg</t>
+  </si>
+  <si>
+    <t>GROC-01</t>
+  </si>
+  <si>
+    <t>8901234567890</t>
+  </si>
+  <si>
+    <t>Grocery</t>
+  </si>
+  <si>
     <t>Bill No</t>
   </si>
   <si>
@@ -135,6 +174,24 @@
   </si>
   <si>
     <t>[{"id":1,"name":"Test Item","qty":4,"price":100}]</t>
+  </si>
+  <si>
+    <t>Test Customer</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>[{"id":3,"name":"Test Product","qty":5,"price":10}]</t>
+  </si>
+  <si>
+    <t>[{"id":10,"name":"Test Product","qty":5,"price":10}]</t>
+  </si>
+  <si>
+    <t>Race Customer</t>
+  </si>
+  <si>
+    <t>[{"id":10,"qty":1}]</t>
   </si>
 </sst>
 </file>
@@ -511,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -683,6 +740,259 @@
         <v>20</v>
       </c>
     </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4">
+        <v>50</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+      <c r="G4">
+        <v>120</v>
+      </c>
+      <c r="H4">
+        <v>80</v>
+      </c>
+      <c r="J4">
+        <v>18</v>
+      </c>
+      <c r="P4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5">
+        <v>50</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+      <c r="G5">
+        <v>120</v>
+      </c>
+      <c r="H5">
+        <v>80</v>
+      </c>
+      <c r="J5">
+        <v>18</v>
+      </c>
+      <c r="P5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6">
+        <v>50</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <v>120</v>
+      </c>
+      <c r="H6">
+        <v>80</v>
+      </c>
+      <c r="J6">
+        <v>18</v>
+      </c>
+      <c r="P6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7">
+        <v>50</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="G7">
+        <v>120</v>
+      </c>
+      <c r="H7">
+        <v>80</v>
+      </c>
+      <c r="J7">
+        <v>18</v>
+      </c>
+      <c r="P7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8">
+        <v>50</v>
+      </c>
+      <c r="F8">
+        <v>100</v>
+      </c>
+      <c r="G8">
+        <v>120</v>
+      </c>
+      <c r="H8">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="P8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9">
+        <v>50</v>
+      </c>
+      <c r="F9">
+        <v>100</v>
+      </c>
+      <c r="G9">
+        <v>120</v>
+      </c>
+      <c r="H9">
+        <v>80</v>
+      </c>
+      <c r="J9">
+        <v>18</v>
+      </c>
+      <c r="P9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10">
+        <v>50</v>
+      </c>
+      <c r="F10">
+        <v>100</v>
+      </c>
+      <c r="G10">
+        <v>120</v>
+      </c>
+      <c r="H10">
+        <v>80</v>
+      </c>
+      <c r="J10">
+        <v>18</v>
+      </c>
+      <c r="P10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11">
+        <v>50</v>
+      </c>
+      <c r="F11">
+        <v>250</v>
+      </c>
+      <c r="G11">
+        <v>280</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -691,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -706,34 +1016,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="H1" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="I1" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="J1" t="s">
         <v>12</v>
       </c>
       <c r="K1" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -741,13 +1051,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="H2">
         <v>400</v>
       </c>
       <c r="K2" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -755,13 +1065,166 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="H3">
         <v>400</v>
       </c>
       <c r="K3" t="s">
-        <v>40</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+      <c r="I4" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
+      </c>
+      <c r="I8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9">
+        <v>100</v>
+      </c>
+      <c r="K9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>10</v>
+      </c>
+      <c r="I11" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H12">
+        <v>100</v>
+      </c>
+      <c r="K12" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement discount coupons, glassmorphism navbar, stock management syncing, and thermal printer compatibility fixes
</commit_message>
<xml_diff>
--- a/master-assist/server/database.xlsx
+++ b/master-assist/server/database.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -143,6 +143,27 @@
     <t>Grocery</t>
   </si>
   <si>
+    <t>WHITE SHOE</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>890935170003</t>
+  </si>
+  <si>
+    <t>P&amp;G</t>
+  </si>
+  <si>
+    <t>shirt large</t>
+  </si>
+  <si>
+    <t>rredyu679</t>
+  </si>
+  <si>
+    <t>Beverages</t>
+  </si>
+  <si>
     <t>Bill No</t>
   </si>
   <si>
@@ -192,6 +213,48 @@
   </si>
   <si>
     <t>[{"id":10,"qty":1}]</t>
+  </si>
+  <si>
+    <t>[{"id":11,"name":"Test Product","qty":5,"price":10}]</t>
+  </si>
+  <si>
+    <t>[{"id":11,"qty":1}]</t>
+  </si>
+  <si>
+    <t>[{"id":12,"name":"Test Product","qty":5,"price":10}]</t>
+  </si>
+  <si>
+    <t>[{"id":12,"qty":1}]</t>
+  </si>
+  <si>
+    <t>[{"id":13,"name":"Test Product","qty":5,"price":10}]</t>
+  </si>
+  <si>
+    <t>[{"id":13,"qty":1}]</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>2026-08-03</t>
+  </si>
+  <si>
+    <t>19:14</t>
+  </si>
+  <si>
+    <t>Walk-in</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>[{"id":11,"name":"WHITE SHOE","qty":1,"price":2999,"originalPrice":2999,"gst":18}]</t>
+  </si>
+  <si>
+    <t>19:17</t>
+  </si>
+  <si>
+    <t>[{"id":11,"name":"WHITE SHOE","qty":2,"price":2999,"originalPrice":2999,"gst":18}]</t>
   </si>
 </sst>
 </file>
@@ -568,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -993,6 +1056,91 @@
         <v>42</v>
       </c>
     </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12">
+        <v>96</v>
+      </c>
+      <c r="F12">
+        <v>2999</v>
+      </c>
+      <c r="G12">
+        <v>2899</v>
+      </c>
+      <c r="H12">
+        <v>1999</v>
+      </c>
+      <c r="I12">
+        <v>10</v>
+      </c>
+      <c r="J12" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M12" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" t="s">
+        <v>28</v>
+      </c>
+      <c r="O12" t="s">
+        <v>20</v>
+      </c>
+      <c r="P12" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13">
+        <v>59</v>
+      </c>
+      <c r="F13">
+        <v>500</v>
+      </c>
+      <c r="G13">
+        <v>500</v>
+      </c>
+      <c r="H13">
+        <v>400</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="K13" t="s">
+        <v>49</v>
+      </c>
+      <c r="N13" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -1001,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1016,34 +1164,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="G1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="H1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I1" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="J1" t="s">
         <v>12</v>
       </c>
       <c r="K1" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1051,13 +1199,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="H2">
         <v>400</v>
       </c>
       <c r="K2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1065,13 +1213,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="H3">
         <v>400</v>
       </c>
       <c r="K3" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1079,7 +1227,7 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F4">
         <v>10</v>
@@ -1088,10 +1236,10 @@
         <v>10</v>
       </c>
       <c r="I4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1099,7 +1247,7 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F5">
         <v>10</v>
@@ -1108,10 +1256,10 @@
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1119,7 +1267,7 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F6">
         <v>10</v>
@@ -1128,10 +1276,10 @@
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1139,7 +1287,7 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F7">
         <v>10</v>
@@ -1148,10 +1296,10 @@
         <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1159,7 +1307,7 @@
         <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F8">
         <v>10</v>
@@ -1168,10 +1316,10 @@
         <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K8" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1179,13 +1327,13 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H9">
         <v>100</v>
       </c>
       <c r="K9" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -1198,7 +1346,7 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F11">
         <v>10</v>
@@ -1207,10 +1355,10 @@
         <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K11" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1218,13 +1366,313 @@
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H12">
         <v>100</v>
       </c>
       <c r="K12" t="s">
-        <v>59</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13">
+        <v>10</v>
+      </c>
+      <c r="H13">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s">
+        <v>62</v>
+      </c>
+      <c r="K13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14">
+        <v>100</v>
+      </c>
+      <c r="K14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="E15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15">
+        <v>10</v>
+      </c>
+      <c r="H15">
+        <v>10</v>
+      </c>
+      <c r="I15" t="s">
+        <v>62</v>
+      </c>
+      <c r="K15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="E16" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16">
+        <v>100</v>
+      </c>
+      <c r="K16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17">
+        <v>10</v>
+      </c>
+      <c r="H17">
+        <v>10</v>
+      </c>
+      <c r="I17" t="s">
+        <v>62</v>
+      </c>
+      <c r="K17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18">
+        <v>100</v>
+      </c>
+      <c r="K18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="E19" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19">
+        <v>10</v>
+      </c>
+      <c r="H19">
+        <v>10</v>
+      </c>
+      <c r="I19" t="s">
+        <v>62</v>
+      </c>
+      <c r="K19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="E20" t="s">
+        <v>65</v>
+      </c>
+      <c r="H20">
+        <v>100</v>
+      </c>
+      <c r="K20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="E21" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21">
+        <v>10</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
+      </c>
+      <c r="I21" t="s">
+        <v>62</v>
+      </c>
+      <c r="K21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="E22" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22">
+        <v>100</v>
+      </c>
+      <c r="K22" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23">
+        <v>2999</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>2999</v>
+      </c>
+      <c r="J23" t="s">
+        <v>77</v>
+      </c>
+      <c r="K23" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24">
+        <v>2999</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>2999</v>
+      </c>
+      <c r="J24" t="s">
+        <v>77</v>
+      </c>
+      <c r="K24" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25">
+        <v>5998</v>
+      </c>
+      <c r="G25">
+        <v>33.34</v>
+      </c>
+      <c r="H25">
+        <v>3998</v>
+      </c>
+      <c r="J25" t="s">
+        <v>77</v>
+      </c>
+      <c r="K25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="E26" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26">
+        <v>10</v>
+      </c>
+      <c r="H26">
+        <v>10</v>
+      </c>
+      <c r="I26" t="s">
+        <v>62</v>
+      </c>
+      <c r="K26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="E27" t="s">
+        <v>65</v>
+      </c>
+      <c r="H27">
+        <v>100</v>
+      </c>
+      <c r="K27" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
design: rebuild Add Item form modal with two panel layout and Select2 searchable dropdowns
</commit_message>
<xml_diff>
--- a/master-assist/server/database.xlsx
+++ b/master-assist/server/database.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -1149,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1675,6 +1675,40 @@
         <v>72</v>
       </c>
     </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="E28" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28">
+        <v>10</v>
+      </c>
+      <c r="H28">
+        <v>10</v>
+      </c>
+      <c r="I28" t="s">
+        <v>62</v>
+      </c>
+      <c r="K28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="E29" t="s">
+        <v>65</v>
+      </c>
+      <c r="H29">
+        <v>100</v>
+      </c>
+      <c r="K29" t="s">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
feat: redesign Item Master modal to side-by-side card layout and integrate dynamic Select2 metadata option creation
</commit_message>
<xml_diff>
--- a/master-assist/server/database.xlsx
+++ b/master-assist/server/database.xlsx
@@ -6,13 +6,20 @@
   <sheets>
     <sheet sheetId="1" name="Items" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Sales" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="brands" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="categories" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="sizes" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="colours" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="hsns" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="units" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="itemNames" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -1149,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1743,6 +1750,201 @@
         <v>72</v>
       </c>
     </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="E32" t="s">
+        <v>61</v>
+      </c>
+      <c r="F32">
+        <v>10</v>
+      </c>
+      <c r="H32">
+        <v>10</v>
+      </c>
+      <c r="I32" t="s">
+        <v>62</v>
+      </c>
+      <c r="K32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="E33" t="s">
+        <v>65</v>
+      </c>
+      <c r="H33">
+        <v>100</v>
+      </c>
+      <c r="K33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>